<commit_message>
update pharmacies (rm cache.sqlite)
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -621,7 +621,7 @@
         <v>88</v>
       </c>
       <c r="F2">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G2">
         <v>36</v>
@@ -657,7 +657,7 @@
         <v>8</v>
       </c>
       <c r="R2">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="S2">
         <v>4</v>
@@ -745,7 +745,7 @@
         <v>88</v>
       </c>
       <c r="F4">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G4">
         <v>36</v>
@@ -781,7 +781,7 @@
         <v>8</v>
       </c>
       <c r="R4">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="S4">
         <v>4</v>
@@ -795,19 +795,19 @@
         <v>22</v>
       </c>
       <c r="B5">
-        <v>56.52318295739349</v>
+        <v>56.50814536340852</v>
       </c>
       <c r="C5">
-        <v>51.46186440677966</v>
+        <v>51.5635593220339</v>
       </c>
       <c r="D5">
-        <v>54.04166666666666</v>
+        <v>54.07065217391305</v>
       </c>
       <c r="E5">
-        <v>54.01420454545455</v>
+        <v>53.98011363636363</v>
       </c>
       <c r="F5">
-        <v>56.22933884297521</v>
+        <v>56.33403361344538</v>
       </c>
       <c r="G5">
         <v>51.95138888888889</v>
@@ -819,7 +819,7 @@
         <v>47.61197916666666</v>
       </c>
       <c r="J5">
-        <v>50.359375</v>
+        <v>50.46875</v>
       </c>
       <c r="K5">
         <v>49.02777777777778</v>
@@ -828,7 +828,7 @@
         <v>51.09090909090909</v>
       </c>
       <c r="M5">
-        <v>51.6078431372549</v>
+        <v>51.69019607843138</v>
       </c>
       <c r="N5">
         <v>23.25</v>
@@ -843,7 +843,7 @@
         <v>53.6875</v>
       </c>
       <c r="R5">
-        <v>59.02798507462686</v>
+        <v>58.87781954887218</v>
       </c>
       <c r="S5">
         <v>46.75</v>
@@ -857,19 +857,19 @@
         <v>23</v>
       </c>
       <c r="B6">
-        <v>14.92707565759796</v>
+        <v>14.92861403160505</v>
       </c>
       <c r="C6">
-        <v>11.12999341242428</v>
+        <v>11.3916932474428</v>
       </c>
       <c r="D6">
-        <v>14.13179567594876</v>
+        <v>14.11720972857136</v>
       </c>
       <c r="E6">
-        <v>11.56604957659507</v>
+        <v>11.56902210218009</v>
       </c>
       <c r="F6">
-        <v>17.04313115478575</v>
+        <v>17.1180558514819</v>
       </c>
       <c r="G6">
         <v>11.20743048231275</v>
@@ -881,7 +881,7 @@
         <v>7.307616484227641</v>
       </c>
       <c r="J6">
-        <v>9.729597656867222</v>
+        <v>10.05303476889024</v>
       </c>
       <c r="K6">
         <v>12.05845550667038</v>
@@ -890,7 +890,7 @@
         <v>10.14597994729484</v>
       </c>
       <c r="M6">
-        <v>12.94399837135091</v>
+        <v>13.19490775146083</v>
       </c>
       <c r="N6">
         <v>28.43999531176708</v>
@@ -905,7 +905,7 @@
         <v>9.7245547088653</v>
       </c>
       <c r="R6">
-        <v>14.04168272694861</v>
+        <v>14.00583673451384</v>
       </c>
       <c r="S6">
         <v>1.848422751068236</v>
@@ -1029,7 +1029,7 @@
         <v>46.25</v>
       </c>
       <c r="R8">
-        <v>48.625</v>
+        <v>48.5</v>
       </c>
       <c r="S8">
         <v>45.375</v>
@@ -1117,7 +1117,7 @@
         <v>57</v>
       </c>
       <c r="F10">
-        <v>64.5</v>
+        <v>65.5</v>
       </c>
       <c r="G10">
         <v>56.125</v>
@@ -1153,7 +1153,7 @@
         <v>62.25</v>
       </c>
       <c r="R10">
-        <v>67.875</v>
+        <v>67.5</v>
       </c>
       <c r="S10">
         <v>47.875</v>
@@ -1200,7 +1200,7 @@
         <v>75</v>
       </c>
       <c r="M11">
-        <v>91</v>
+        <v>94.5</v>
       </c>
       <c r="N11">
         <v>73</v>
@@ -1241,7 +1241,7 @@
         <v>83</v>
       </c>
       <c r="F12">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G12">
         <v>32</v>
@@ -1277,7 +1277,7 @@
         <v>8</v>
       </c>
       <c r="R12">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="S12">
         <v>4</v>
@@ -1427,7 +1427,7 @@
         <v>2047.309793814433</v>
       </c>
       <c r="F15">
-        <v>2463.78962264151</v>
+        <v>2502.155188679245</v>
       </c>
       <c r="G15">
         <v>6979.627272727273</v>
@@ -1463,7 +1463,7 @@
         <v>8764.65</v>
       </c>
       <c r="R15">
-        <v>2861.016033755274</v>
+        <v>2863.366666666666</v>
       </c>
       <c r="S15">
         <v>35973.725</v>
@@ -1489,7 +1489,7 @@
         <v>2052.190647588246</v>
       </c>
       <c r="F16">
-        <v>3983.459917627142</v>
+        <v>3983.418649344369</v>
       </c>
       <c r="G16">
         <v>12889.55368946111</v>
@@ -1525,7 +1525,7 @@
         <v>11519.31585799261</v>
       </c>
       <c r="R16">
-        <v>4050.045976532855</v>
+        <v>4048.728775312715</v>
       </c>
       <c r="S16">
         <v>43539.16479837116</v>
@@ -1613,7 +1613,7 @@
         <v>841.2</v>
       </c>
       <c r="F18">
-        <v>845.5749999999999</v>
+        <v>848.025</v>
       </c>
       <c r="G18">
         <v>971</v>
@@ -1649,7 +1649,7 @@
         <v>1215.825</v>
       </c>
       <c r="R18">
-        <v>857</v>
+        <v>871.1</v>
       </c>
       <c r="S18">
         <v>3663.95</v>
@@ -1675,7 +1675,7 @@
         <v>1458.9</v>
       </c>
       <c r="F19">
-        <v>1316.55</v>
+        <v>1348.75</v>
       </c>
       <c r="G19">
         <v>1668.65</v>
@@ -1737,7 +1737,7 @@
         <v>2303.45</v>
       </c>
       <c r="F20">
-        <v>2056.45</v>
+        <v>2077.575</v>
       </c>
       <c r="G20">
         <v>4218.049999999999</v>
@@ -1923,7 +1923,7 @@
         <v>222.9242268041237</v>
       </c>
       <c r="F23">
-        <v>228.3584905660377</v>
+        <v>232.1754716981132</v>
       </c>
       <c r="G23">
         <v>548.7465909090909</v>
@@ -1959,7 +1959,7 @@
         <v>818.8500000000001</v>
       </c>
       <c r="R23">
-        <v>260.0789029535865</v>
+        <v>260.3430379746835</v>
       </c>
       <c r="S23">
         <v>2296.675</v>
@@ -1985,7 +1985,7 @@
         <v>256.549318513439</v>
       </c>
       <c r="F24">
-        <v>302.8297212457006</v>
+        <v>303.2047153253245</v>
       </c>
       <c r="G24">
         <v>1021.255363266083</v>
@@ -2021,7 +2021,7 @@
         <v>1228.265118042518</v>
       </c>
       <c r="R24">
-        <v>300.6403894860383</v>
+        <v>300.4794939350726</v>
       </c>
       <c r="S24">
         <v>2365.057016402212</v>
@@ -2109,7 +2109,7 @@
         <v>101.2</v>
       </c>
       <c r="F26">
-        <v>104.375</v>
+        <v>105.15</v>
       </c>
       <c r="G26">
         <v>108.3</v>
@@ -2145,7 +2145,7 @@
         <v>127.825</v>
       </c>
       <c r="R26">
-        <v>98.5</v>
+        <v>98.7</v>
       </c>
       <c r="S26">
         <v>415.475</v>
@@ -2171,7 +2171,7 @@
         <v>160.5</v>
       </c>
       <c r="F27">
-        <v>149.9</v>
+        <v>150.8</v>
       </c>
       <c r="G27">
         <v>180.1</v>
@@ -2233,7 +2233,7 @@
         <v>246.175</v>
       </c>
       <c r="F28">
-        <v>232.55</v>
+        <v>236.175</v>
       </c>
       <c r="G28">
         <v>374.025</v>

</xml_diff>

<commit_message>
sort index so that <20 is on top
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -3984,385 +3984,385 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>Number of people giving birth aged 20-24</t>
+          <t>Number of people giving birth aged &lt;20</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>400</v>
+        <v>90</v>
       </c>
       <c r="C56" t="n">
-        <v>422</v>
+        <v>146</v>
       </c>
       <c r="D56" t="n">
-        <v>647</v>
+        <v>120</v>
       </c>
       <c r="E56" t="n">
-        <v>463</v>
+        <v>109</v>
       </c>
       <c r="F56" t="n">
-        <v>1276</v>
+        <v>299</v>
       </c>
       <c r="G56" t="n">
-        <v>361</v>
+        <v>78</v>
       </c>
       <c r="H56" t="n">
-        <v>318</v>
+        <v>84</v>
       </c>
       <c r="I56" t="n">
-        <v>367</v>
+        <v>82</v>
       </c>
       <c r="J56" t="n">
-        <v>176</v>
+        <v>46</v>
       </c>
       <c r="K56" t="n">
-        <v>460</v>
+        <v>118</v>
       </c>
       <c r="L56" t="n">
-        <v>82</v>
+        <v>10</v>
       </c>
       <c r="M56" t="n">
-        <v>397</v>
+        <v>80</v>
       </c>
       <c r="N56" t="n">
-        <v>157</v>
+        <v>60</v>
       </c>
       <c r="O56" t="n">
-        <v>221</v>
+        <v>46</v>
       </c>
       <c r="P56" t="n">
-        <v>919</v>
+        <v>211</v>
       </c>
       <c r="Q56" t="n">
-        <v>95</v>
+        <v>23</v>
       </c>
       <c r="R56" t="n">
-        <v>591</v>
+        <v>120</v>
       </c>
       <c r="S56" t="n">
-        <v>46</v>
+        <v>3</v>
       </c>
       <c r="T56" t="n">
-        <v>154</v>
+        <v>49</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>Number of people giving birth aged 25-29</t>
+          <t>Number of people giving birth aged 20-24</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>932</v>
+        <v>400</v>
       </c>
       <c r="C57" t="n">
-        <v>861</v>
+        <v>422</v>
       </c>
       <c r="D57" t="n">
-        <v>1636</v>
+        <v>647</v>
       </c>
       <c r="E57" t="n">
-        <v>1051</v>
+        <v>463</v>
       </c>
       <c r="F57" t="n">
-        <v>2240</v>
+        <v>1276</v>
       </c>
       <c r="G57" t="n">
-        <v>584</v>
+        <v>361</v>
       </c>
       <c r="H57" t="n">
-        <v>456</v>
+        <v>318</v>
       </c>
       <c r="I57" t="n">
-        <v>658</v>
+        <v>367</v>
       </c>
       <c r="J57" t="n">
-        <v>365</v>
+        <v>176</v>
       </c>
       <c r="K57" t="n">
-        <v>639</v>
+        <v>460</v>
       </c>
       <c r="L57" t="n">
+        <v>82</v>
+      </c>
+      <c r="M57" t="n">
+        <v>397</v>
+      </c>
+      <c r="N57" t="n">
+        <v>157</v>
+      </c>
+      <c r="O57" t="n">
+        <v>221</v>
+      </c>
+      <c r="P57" t="n">
+        <v>919</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>95</v>
+      </c>
+      <c r="R57" t="n">
+        <v>591</v>
+      </c>
+      <c r="S57" t="n">
+        <v>46</v>
+      </c>
+      <c r="T57" t="n">
         <v>154</v>
-      </c>
-      <c r="M57" t="n">
-        <v>827</v>
-      </c>
-      <c r="N57" t="n">
-        <v>184</v>
-      </c>
-      <c r="O57" t="n">
-        <v>370</v>
-      </c>
-      <c r="P57" t="n">
-        <v>1536</v>
-      </c>
-      <c r="Q57" t="n">
-        <v>179</v>
-      </c>
-      <c r="R57" t="n">
-        <v>1733</v>
-      </c>
-      <c r="S57" t="n">
-        <v>81</v>
-      </c>
-      <c r="T57" t="n">
-        <v>247</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>Number of people giving birth aged 30-34</t>
+          <t>Number of people giving birth aged 25-29</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>1957</v>
+        <v>932</v>
       </c>
       <c r="C58" t="n">
-        <v>1046</v>
+        <v>861</v>
       </c>
       <c r="D58" t="n">
-        <v>2505</v>
+        <v>1636</v>
       </c>
       <c r="E58" t="n">
-        <v>1787</v>
+        <v>1051</v>
       </c>
       <c r="F58" t="n">
-        <v>2651</v>
+        <v>2240</v>
       </c>
       <c r="G58" t="n">
-        <v>657</v>
+        <v>584</v>
       </c>
       <c r="H58" t="n">
-        <v>444</v>
+        <v>456</v>
       </c>
       <c r="I58" t="n">
-        <v>650</v>
+        <v>658</v>
       </c>
       <c r="J58" t="n">
-        <v>508</v>
+        <v>365</v>
       </c>
       <c r="K58" t="n">
-        <v>714</v>
+        <v>639</v>
       </c>
       <c r="L58" t="n">
-        <v>220</v>
+        <v>154</v>
       </c>
       <c r="M58" t="n">
-        <v>1217</v>
+        <v>827</v>
       </c>
       <c r="N58" t="n">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="O58" t="n">
-        <v>489</v>
+        <v>370</v>
       </c>
       <c r="P58" t="n">
-        <v>1784</v>
+        <v>1536</v>
       </c>
       <c r="Q58" t="n">
-        <v>154</v>
+        <v>179</v>
       </c>
       <c r="R58" t="n">
-        <v>2872</v>
+        <v>1733</v>
       </c>
       <c r="S58" t="n">
-        <v>109</v>
+        <v>81</v>
       </c>
       <c r="T58" t="n">
-        <v>226</v>
+        <v>247</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>Number of people giving birth aged 35-39</t>
+          <t>Number of people giving birth aged 30-34</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>1280</v>
+        <v>1957</v>
       </c>
       <c r="C59" t="n">
-        <v>568</v>
+        <v>1046</v>
       </c>
       <c r="D59" t="n">
-        <v>1271</v>
+        <v>2505</v>
       </c>
       <c r="E59" t="n">
-        <v>1099</v>
+        <v>1787</v>
       </c>
       <c r="F59" t="n">
-        <v>1301</v>
+        <v>2651</v>
       </c>
       <c r="G59" t="n">
-        <v>300</v>
+        <v>657</v>
       </c>
       <c r="H59" t="n">
-        <v>213</v>
+        <v>444</v>
       </c>
       <c r="I59" t="n">
-        <v>345</v>
+        <v>650</v>
       </c>
       <c r="J59" t="n">
-        <v>237</v>
+        <v>508</v>
       </c>
       <c r="K59" t="n">
-        <v>356</v>
+        <v>714</v>
       </c>
       <c r="L59" t="n">
-        <v>89</v>
+        <v>220</v>
       </c>
       <c r="M59" t="n">
-        <v>653</v>
+        <v>1217</v>
       </c>
       <c r="N59" t="n">
-        <v>94</v>
+        <v>188</v>
       </c>
       <c r="O59" t="n">
-        <v>225</v>
+        <v>489</v>
       </c>
       <c r="P59" t="n">
-        <v>786</v>
+        <v>1784</v>
       </c>
       <c r="Q59" t="n">
-        <v>63</v>
+        <v>154</v>
       </c>
       <c r="R59" t="n">
-        <v>1664</v>
+        <v>2872</v>
       </c>
       <c r="S59" t="n">
-        <v>43</v>
+        <v>109</v>
       </c>
       <c r="T59" t="n">
-        <v>115</v>
+        <v>226</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>Number of people giving birth aged 40+</t>
+          <t>Number of people giving birth aged 35-39</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>294</v>
+        <v>1280</v>
       </c>
       <c r="C60" t="n">
-        <v>104</v>
+        <v>568</v>
       </c>
       <c r="D60" t="n">
-        <v>274</v>
+        <v>1271</v>
       </c>
       <c r="E60" t="n">
-        <v>227</v>
+        <v>1099</v>
       </c>
       <c r="F60" t="n">
-        <v>285</v>
+        <v>1301</v>
       </c>
       <c r="G60" t="n">
-        <v>66</v>
+        <v>300</v>
       </c>
       <c r="H60" t="n">
-        <v>45</v>
+        <v>213</v>
       </c>
       <c r="I60" t="n">
-        <v>55</v>
+        <v>345</v>
       </c>
       <c r="J60" t="n">
-        <v>55</v>
+        <v>237</v>
       </c>
       <c r="K60" t="n">
-        <v>79</v>
+        <v>356</v>
       </c>
       <c r="L60" t="n">
-        <v>23</v>
+        <v>89</v>
       </c>
       <c r="M60" t="n">
-        <v>145</v>
+        <v>653</v>
       </c>
       <c r="N60" t="n">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="O60" t="n">
-        <v>46</v>
+        <v>225</v>
       </c>
       <c r="P60" t="n">
-        <v>175</v>
+        <v>786</v>
       </c>
       <c r="Q60" t="n">
-        <v>11</v>
+        <v>63</v>
       </c>
       <c r="R60" t="n">
-        <v>373</v>
+        <v>1664</v>
       </c>
       <c r="S60" t="n">
-        <v>12</v>
+        <v>43</v>
       </c>
       <c r="T60" t="n">
-        <v>23</v>
+        <v>115</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>Number of people giving birth aged &lt;20</t>
+          <t>Number of people giving birth aged 40+</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>90</v>
+        <v>294</v>
       </c>
       <c r="C61" t="n">
-        <v>146</v>
+        <v>104</v>
       </c>
       <c r="D61" t="n">
-        <v>120</v>
+        <v>274</v>
       </c>
       <c r="E61" t="n">
-        <v>109</v>
+        <v>227</v>
       </c>
       <c r="F61" t="n">
-        <v>299</v>
+        <v>285</v>
       </c>
       <c r="G61" t="n">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="H61" t="n">
-        <v>84</v>
+        <v>45</v>
       </c>
       <c r="I61" t="n">
-        <v>82</v>
+        <v>55</v>
       </c>
       <c r="J61" t="n">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="K61" t="n">
-        <v>118</v>
+        <v>79</v>
       </c>
       <c r="L61" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="M61" t="n">
-        <v>80</v>
+        <v>145</v>
       </c>
       <c r="N61" t="n">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="O61" t="n">
         <v>46</v>
       </c>
       <c r="P61" t="n">
-        <v>211</v>
+        <v>175</v>
       </c>
       <c r="Q61" t="n">
+        <v>11</v>
+      </c>
+      <c r="R61" t="n">
+        <v>373</v>
+      </c>
+      <c r="S61" t="n">
+        <v>12</v>
+      </c>
+      <c r="T61" t="n">
         <v>23</v>
-      </c>
-      <c r="R61" t="n">
-        <v>120</v>
-      </c>
-      <c r="S61" t="n">
-        <v>3</v>
-      </c>
-      <c r="T61" t="n">
-        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>